<commit_message>
Align Replus glazing order and reevaluate downstream function compatibility
</commit_message>
<xml_diff>
--- a/changes/replus-runtime-v5/candidates/RPL_BATH.xlsx
+++ b/changes/replus-runtime-v5/candidates/RPL_BATH.xlsx
@@ -1291,7 +1291,7 @@
         <v>USER_APPLICATION_POLICY</v>
       </c>
       <c r="F3" t="str">
-        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
       </c>
     </row>
     <row r="4">
@@ -1311,7 +1311,7 @@
         <v>USER_APPLICATION_POLICY</v>
       </c>
       <c r="F4" t="str">
-        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
       </c>
     </row>
     <row r="5">
@@ -1329,7 +1329,7 @@
         <v>OFFICIAL_SOURCE_REVIEW</v>
       </c>
       <c r="F5" t="str">
-        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
       </c>
     </row>
     <row r="6">
@@ -1349,7 +1349,7 @@
         <v>OFFICIAL_SOURCE_REVIEW</v>
       </c>
       <c r="F6" t="str">
-        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
       </c>
     </row>
     <row r="7">
@@ -1367,7 +1367,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F7" t="str">
-        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
       </c>
     </row>
     <row r="8">
@@ -1387,7 +1387,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F8" t="str">
-        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
       </c>
     </row>
     <row r="9">
@@ -1407,7 +1407,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F9" t="str">
-        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
       </c>
     </row>
     <row r="10">
@@ -1427,7 +1427,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F10" t="str">
-        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
       </c>
     </row>
     <row r="11">
@@ -1447,7 +1447,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F11" t="str">
-        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
       </c>
     </row>
     <row r="12">
@@ -1467,7 +1467,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F12" t="str">
-        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
       </c>
     </row>
     <row r="13">
@@ -1485,7 +1485,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F13" t="str">
-        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
       </c>
     </row>
     <row r="14">
@@ -1503,7 +1503,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F14" t="str">
-        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
       </c>
     </row>
     <row r="15">
@@ -1523,7 +1523,7 @@
         <v>USER_PRESENTATION_POLICY</v>
       </c>
       <c r="F15" t="str">
-        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
       </c>
     </row>
     <row r="16">
@@ -1541,7 +1541,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F16" t="str">
-        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
       </c>
     </row>
     <row r="17">
@@ -1561,7 +1561,7 @@
         <v>USER_PRESENTATION_POLICY</v>
       </c>
       <c r="F17" t="str">
-        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
       </c>
     </row>
     <row r="18">
@@ -1579,7 +1579,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F18" t="str">
-        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
       </c>
     </row>
     <row r="19">
@@ -1597,7 +1597,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F19" t="str">
-        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
       </c>
     </row>
     <row r="20">
@@ -1615,7 +1615,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F20" t="str">
-        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
       </c>
     </row>
     <row r="21">
@@ -1629,13 +1629,13 @@
         <v>frame_type,installation_region,window_type</v>
       </c>
       <c r="D21" t="str" s="185">
-        <v>{"label": "ガラス種類", "group": "glazing", "internal": false}</v>
+        <v>{"label": "ガラス種類", "group": "glazing", "internal": false, "rank": 1}</v>
       </c>
       <c r="E21" t="str" s="186">
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F21" t="str">
-        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
       </c>
     </row>
     <row r="22">
@@ -1646,16 +1646,16 @@
         <v>glass</v>
       </c>
       <c r="C22" t="str" s="185">
-        <v>frame_type,glass_category,installation_region,window_type</v>
+        <v>frame_type,glass_appearance,glass_category,installation_region,window_type</v>
       </c>
       <c r="D22" t="str" s="185">
-        <v>{"label": "ガラス詳細・Low-E仕様", "group": "glazing", "internal": false}</v>
+        <v>{"label": "ガラス詳細・Low-E仕様", "group": "glazing", "internal": false, "rank": 3}</v>
       </c>
       <c r="E22" t="str" s="186">
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F22" t="str">
-        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
       </c>
     </row>
     <row r="23">
@@ -1675,7 +1675,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F23" t="str">
-        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
       </c>
     </row>
     <row r="24">
@@ -1695,7 +1695,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F24" t="str">
-        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
       </c>
     </row>
     <row r="25">
@@ -1715,7 +1715,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F25" t="str">
-        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
       </c>
     </row>
     <row r="26">
@@ -1726,16 +1726,16 @@
         <v>glass_function</v>
       </c>
       <c r="C26" t="str" s="185">
-        <v>glass_category,glass,window_type</v>
+        <v>glass_category,glass_appearance,glass,window_type</v>
       </c>
       <c r="D26" t="str" s="185">
-        <v>{"label": "ガラス追加機能", "group": "glazing", "internal": false}</v>
+        <v>{"label": "ガラス追加機能", "group": "glazing", "internal": false, "rank": 4}</v>
       </c>
       <c r="E26" t="str" s="186">
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F26" t="str">
-        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
       </c>
     </row>
     <row r="27">
@@ -1746,16 +1746,16 @@
         <v>glass_appearance</v>
       </c>
       <c r="C27" t="str" s="185">
-        <v>glass,glass_function</v>
+        <v>glass_category</v>
       </c>
       <c r="D27" t="str" s="185">
-        <v>{"label": "ガラス仕上げ・目隠し", "group": "glazing", "internal": false}</v>
+        <v>{"label": "ガラス種", "group": "glazing", "internal": false, "rank": 2}</v>
       </c>
       <c r="E27" t="str" s="186">
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F27" t="str">
-        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
       </c>
     </row>
     <row r="28">
@@ -1775,7 +1775,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F28" t="str">
-        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
       </c>
     </row>
     <row r="29">
@@ -1795,7 +1795,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F29" t="str">
-        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
       </c>
     </row>
     <row r="30">
@@ -1815,7 +1815,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F30" t="str">
-        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
       </c>
     </row>
     <row r="31">
@@ -1835,7 +1835,7 @@
         <v>USER_PRESENTATION_POLICY</v>
       </c>
       <c r="F31" t="str">
-        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
       </c>
     </row>
     <row r="32">
@@ -1853,7 +1853,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F32" t="str">
-        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
       </c>
     </row>
     <row r="33">
@@ -1873,7 +1873,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F33" t="str">
-        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
       </c>
     </row>
     <row r="34">
@@ -1893,7 +1893,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F34" t="str">
-        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
       </c>
     </row>
     <row r="35">
@@ -1913,7 +1913,7 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F35" t="str">
-        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
       </c>
     </row>
     <row r="36">
@@ -1933,7 +1933,67 @@
         <v>UI_PRESENTATION</v>
       </c>
       <c r="F36" t="str">
-        <v>REPLUS_HIDE_DERIVED_CONFIRMATIONS_V12_20261014</v>
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>FIELD_PATCH</v>
+      </c>
+      <c r="B37" t="str">
+        <v>glass_appearance</v>
+      </c>
+      <c r="C37" t="str">
+        <v>glass_category</v>
+      </c>
+      <c r="D37" t="str">
+        <v>{"key": "glass_appearance", "displayLabel": "ガラス種", "dataType": "ENUM", "displayOrder": 710, "required": false, "autoSelectSingle": false, "parentFields": ["glass_category"], "selector": {"glass_category": {"$exists": true}}, "choices": [{"value": "MILKY", "displayLabel": "乳白", "selector": {"glass_category": {"$exists": true}}, "evidenceIds": ["EV-V8-GLASS-DIAGRAM"], "metadata": {"manualCheck": true, "estimateConfirmationRequired": true}, "displayOrder": 4}, {"value": "CLEAR", "displayLabel": "透明", "selector": {"glass_category": {"$exists": true}}, "evidenceIds": ["EV-V8-GLASS-DIAGRAM"], "metadata": {"manualCheck": true, "estimateConfirmationRequired": true}, "displayOrder": 1}, {"value": "OBSCURE", "displayLabel": "型板", "selector": {"glass_category": {"$exists": true}}, "evidenceIds": ["EV-V8-GLASS-DIAGRAM"], "metadata": {"manualCheck": true, "estimateConfirmationRequired": true}, "displayOrder": 2}, {"value": "FROST", "displayLabel": "フロスト", "selector": {"glass_category": {"$exists": true}}, "evidenceIds": ["EV-V8-GLASS-DIAGRAM"], "metadata": {"manualCheck": true, "estimateConfirmationRequired": true}, "displayOrder": 3}]}</v>
+      </c>
+      <c r="E37" t="str">
+        <v>USER_FLOW_POLICY_WITH_EXISTING_EVIDENCE</v>
+      </c>
+      <c r="F37" t="str">
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>FIELD_PATCH</v>
+      </c>
+      <c r="B38" t="str">
+        <v>glass</v>
+      </c>
+      <c r="C38" t="str">
+        <v>frame_type,glass_appearance,glass_category,installation_region,window_type</v>
+      </c>
+      <c r="D38" t="str">
+        <v>{"key": "glass", "displayLabel": "ガラス詳細・Low-E仕様", "dataType": "ENUM", "displayOrder": 720, "choices": [{"value": "BATH-GL-GENERAL", "displayLabel": "一般複層ガラス", "evidenceIds": ["BATH-EV-004,010"], "selector": {"window_type": {"$exists": true}, "frame_type": "BATH-STD", "glass_category": "GENERAL_DOUBLE"}, "metadata": {"manualCheck": true}}, {"value": "BATH-GL-LOWE-CLEAR", "displayLabel": "Low-E複層 クリア", "evidenceIds": ["BATH-EV-004,010"], "selector": {"window_type": {"$exists": true}, "frame_type": {"$exists": true}, "glass_category": "LOW_E_DOUBLE"}, "metadata": {"manualCheck": true}}, {"value": "BATH-GL-LOWE-GREEN", "displayLabel": "Low-E複層 グリーン", "evidenceIds": ["BATH-EV-004,010"], "selector": {"window_type": {"$exists": true}, "frame_type": {"$exists": true}, "glass_category": "LOW_E_DOUBLE"}, "metadata": {"manualCheck": true}}, {"value": "BATH-GL-LOWE-HS", "displayLabel": "Low-E複層 グリーン（高遮熱仕様）", "evidenceIds": ["BATH-EV-004,010"], "selector": {"window_type": {"$exists": true}, "frame_type": {"$exists": true}, "glass_category": "LOW_E_DOUBLE"}, "metadata": {"manualCheck": true}}, {"value": "BATH-GL-LOWE-BRONZE", "displayLabel": "Low-E複層 ブロンズ", "evidenceIds": ["BATH-EV-010"], "selector": {"window_type": {"$exists": true}, "frame_type": {"$exists": true}, "installation_region": {"$in": ["北海道", "東北"]}, "glass_category": "LOW_E_DOUBLE"}, "metadata": {"manualCheck": true}}, {"value": "BATH-GL-T-CC", "displayLabel": "トリプル クリア×クリア", "evidenceIds": ["BATH-EV-004,010"], "selector": {"window_type": "RPL_BATH_DHFS", "frame_type": {"$exists": true}, "glass_category": "TRIPLE"}, "metadata": {"manualCheck": true}}, {"value": "BATH-GL-T-GG", "displayLabel": "トリプル グリーン×グリーン", "evidenceIds": ["BATH-EV-004,010"], "selector": {"window_type": "RPL_BATH_DHFS", "frame_type": {"$exists": true}, "glass_category": "TRIPLE"}, "metadata": {"manualCheck": true}}, {"value": "BATH-GL-T-CG", "displayLabel": "トリプル クリア×グリーン", "evidenceIds": ["BATH-EV-010"], "selector": {"window_type": "RPL_BATH_DHFS", "frame_type": {"$exists": true}, "glass_category": "TRIPLE"}, "metadata": {"manualCheck": true}}, {"value": "BATH-GL-T-CB", "displayLabel": "トリプル クリア×ブロンズ", "evidenceIds": ["BATH-EV-010"], "selector": {"window_type": "RPL_BATH_DHFS", "frame_type": {"$exists": true}, "installation_region": {"$in": ["北海道", "東北"]}, "glass_category": "TRIPLE"}, "metadata": {"manualCheck": true}}], "required": false, "autoSelectSingle": false, "parentFields": ["frame_type", "glass_appearance", "glass_category", "installation_region", "window_type"], "selector": {"glass_category": {"$exists": true}}}</v>
+      </c>
+      <c r="E38" t="str">
+        <v>USER_FLOW_POLICY_WITH_EXISTING_EVIDENCE</v>
+      </c>
+      <c r="F38" t="str">
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>FIELD_PATCH</v>
+      </c>
+      <c r="B39" t="str">
+        <v>glass_function</v>
+      </c>
+      <c r="C39" t="str">
+        <v>glass_category,glass_appearance,glass,window_type</v>
+      </c>
+      <c r="D39" t="str">
+        <v>{"key": "glass_function", "displayLabel": "ガラス追加機能", "dataType": "ENUM", "displayOrder": 730, "required": false, "autoSelectSingle": false, "parentFields": ["glass_category", "glass_appearance", "glass", "window_type"], "selector": {"glass": {"$exists": true}}, "choices": [{"value": "NONE", "displayLabel": "なし（標準）", "selector": {"all": [{"glass_category": "GENERAL_DOUBLE", "glass": {"$exists": true}}, {"not": {"glass_appearance": "MILKY"}}]}, "evidenceIds": ["EV-V8-GLASS-DIAGRAM"], "metadata": {"manualCheck": false, "estimateConfirmationRequired": false}, "displayOrder": 1}, {"value": "SAFETY", "displayLabel": "安全合わせ", "selector": {"all": [{"glass_category": "GENERAL_DOUBLE", "glass": {"$exists": true}}, {"not": {"glass_appearance": "MILKY"}}]}, "evidenceIds": ["EV-V8-GLASS-DIAGRAM"], "metadata": {"manualCheck": true, "estimateConfirmationRequired": true}, "displayOrder": 2}, {"value": "DISASTER", "displayLabel": "防災安全合わせ", "selector": {"all": [{"glass_category": "GENERAL_DOUBLE", "glass": {"$exists": true}}, {"not": {"glass_appearance": "MILKY"}}]}, "evidenceIds": ["EV-V8-GLASS-DIAGRAM"], "metadata": {"manualCheck": true, "estimateConfirmationRequired": true}, "displayOrder": 3}, {"value": "MILKY", "displayLabel": "安全合わせ乳白タイプ", "selector": {"all": [{"glass_category": "GENERAL_DOUBLE", "glass": {"$exists": true}}, {"glass_appearance": "MILKY"}]}, "evidenceIds": ["EV-V8-GLASS-DIAGRAM"], "metadata": {"manualCheck": true, "estimateConfirmationRequired": true}, "displayOrder": 4}, {"value": "GRID", "displayLabel": "格子入り", "selector": {"all": [{"glass_category": "GENERAL_DOUBLE", "glass": {"$exists": true}}, {"not": {"glass_appearance": "MILKY"}}]}, "evidenceIds": ["EV-V8-GLASS-DIAGRAM"], "metadata": {"manualCheck": true, "estimateConfirmationRequired": true}, "displayOrder": 5}, {"value": "BLIND", "displayLabel": "ブラインドインPG", "selector": {"all": [{"glass_category": "GENERAL_DOUBLE", "glass": {"$exists": true}}, {"not": {"glass_appearance": "MILKY"}}]}, "evidenceIds": ["EV-V8-GLASS-DIAGRAM"], "metadata": {"manualCheck": true, "estimateConfirmationRequired": true}, "displayOrder": 6}, {"value": "NONE", "displayLabel": "なし（標準）", "selector": {"all": [{"glass_category": "LOW_E_DOUBLE", "glass": {"$exists": true}}, {"not": {"glass_appearance": "MILKY"}}]}, "evidenceIds": ["EV-V8-GLASS-DIAGRAM"], "metadata": {"manualCheck": false, "estimateConfirmationRequired": false}, "displayOrder": 1}, {"value": "SAFETY", "displayLabel": "安全合わせ", "selector": {"all": [{"glass_category": "LOW_E_DOUBLE", "glass": {"$exists": true}}, {"not": {"glass_appearance": "MILKY"}}]}, "evidenceIds": ["EV-V8-GLASS-DIAGRAM"], "metadata": {"manualCheck": true, "estimateConfirmationRequired": true}, "displayOrder": 2}, {"value": "DISASTER", "displayLabel": "防災安全合わせ", "selector": {"all": [{"glass_category": "LOW_E_DOUBLE", "glass": {"$exists": true}}, {"not": {"glass_appearance": "MILKY"}}]}, "evidenceIds": ["EV-V8-GLASS-DIAGRAM"], "metadata": {"manualCheck": true, "estimateConfirmationRequired": true}, "displayOrder": 3}, {"value": "MILKY", "displayLabel": "安全合わせ乳白タイプ", "selector": {"all": [{"glass_category": "LOW_E_DOUBLE", "glass": {"$exists": true}}, {"glass_appearance": "MILKY"}]}, "evidenceIds": ["EV-V8-GLASS-DIAGRAM"], "metadata": {"manualCheck": true, "estimateConfirmationRequired": true}, "displayOrder": 4}, {"value": "GRID", "displayLabel": "格子入り", "selector": {"all": [{"glass_category": "LOW_E_DOUBLE", "glass": {"$exists": true}}, {"not": {"glass_appearance": "MILKY"}}]}, "evidenceIds": ["EV-V8-GLASS-DIAGRAM"], "metadata": {"manualCheck": true, "estimateConfirmationRequired": true}, "displayOrder": 5}, {"value": "BLIND", "displayLabel": "ブラインドインPG", "selector": {"all": [{"glass_category": "LOW_E_DOUBLE", "glass": {"$exists": true}}, {"not": {"glass_appearance": "MILKY"}}]}, "evidenceIds": ["EV-V8-GLASS-DIAGRAM"], "metadata": {"manualCheck": true, "estimateConfirmationRequired": true}, "displayOrder": 6}, {"value": "NONE", "displayLabel": "なし（標準）", "selector": {"all": [{"glass_category": "TRIPLE", "glass": {"$exists": true}}, {"not": {"glass_appearance": "MILKY"}}]}, "evidenceIds": ["EV-V8-GLASS-DIAGRAM"], "metadata": {"manualCheck": false, "estimateConfirmationRequired": false}, "displayOrder": 1}, {"value": "SAFETY", "displayLabel": "安全合わせ", "selector": {"all": [{"glass_category": "TRIPLE", "glass": {"$exists": true}}, {"not": {"glass_appearance": "MILKY"}}]}, "evidenceIds": ["EV-V8-GLASS-DIAGRAM"], "metadata": {"manualCheck": true, "estimateConfirmationRequired": true}, "displayOrder": 2}, {"value": "DISASTER", "displayLabel": "防災安全合わせ", "selector": {"all": [{"glass_category": "TRIPLE", "glass": {"$exists": true}}, {"not": {"glass_appearance": "MILKY"}}]}, "evidenceIds": ["EV-V8-GLASS-DIAGRAM"], "metadata": {"manualCheck": true, "estimateConfirmationRequired": true}, "displayOrder": 3}, {"value": "MILKY", "displayLabel": "安全合わせ乳白タイプ", "selector": {"all": [{"glass_category": "TRIPLE", "glass": {"$exists": true}}, {"glass_appearance": "MILKY"}]}, "evidenceIds": ["EV-V8-GLASS-DIAGRAM"], "metadata": {"manualCheck": true, "estimateConfirmationRequired": true}, "displayOrder": 4}, {"value": "THIN", "displayLabel": "特殊薄板合わせ", "selector": {"all": [{"glass_category": "TRIPLE", "glass": {"$exists": true}}, {"not": {"glass_appearance": "MILKY"}}]}, "evidenceIds": ["EV-V8-GLASS-DIAGRAM"], "metadata": {"manualCheck": true, "estimateConfirmationRequired": true}, "displayOrder": 7}]}</v>
+      </c>
+      <c r="E39" t="str">
+        <v>USER_FLOW_POLICY_WITH_EXISTING_EVIDENCE</v>
+      </c>
+      <c r="F39" t="str">
+        <v>REPLUS_GLASS_APPEARANCE_FIRST_V13_20261014</v>
       </c>
     </row>
   </sheetData>

</xml_diff>